<commit_message>
feat(scheduler): English weekly pre-assigned teachers + availability check
- Add _ENG_WEEKLY_PREASSIGNED constant with Jo's B3:K27 assignments (25 classes × 6 blocks)
- Add _load_english_weekly_from_wb(): reads "English Weekly" Excel sheet if present
- Rewrite assign_english_weekly(): 3-mode priority:
    1. Excel "English Weekly" sheet (if filled)
    2. _ENG_WEEKLY_PREASSIGNED hard-coded constant (fallback for this term)
    3. Auto-assign legacy algorithm (fallback if no pre-assignments)
- Add teacher availability check (B44): warn if pre-assigned teacher unavailable on class day
- Net shortfall validation now inside assign_english_weekly() (returns warnings list)
- Add "English Weekly" input sheet to Planning for Timetable.xlsx + V4 Template

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Planning for Timetable V4 Template.xlsx
+++ b/data/input/Planning for Timetable V4 Template.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teacher Availability" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Class list answer" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Net Teachers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="English Weekly" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -87,7 +88,7 @@
       <color rgb="00888888"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -129,6 +130,11 @@
         <fgColor rgb="0015803D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -142,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -177,6 +183,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -4858,4 +4867,996 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="10" min="1" max="1"/>
+    <col width="20" customWidth="1" style="10" min="2" max="2"/>
+    <col width="20" customWidth="1" style="10" min="3" max="3"/>
+    <col width="20" customWidth="1" style="10" min="4" max="4"/>
+    <col width="20" customWidth="1" style="10" min="5" max="5"/>
+    <col width="20" customWidth="1" style="10" min="6" max="6"/>
+    <col width="20" customWidth="1" style="10" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Class Code</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>T2025C wk1-5</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>T2025C wk6-10</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>T2025C wk11-15</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>T2026A wk1-5</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>T2026A wk6-10</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>T2026A wk11-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t># Edit teacher names below. System uses this sheet if filled; otherwise uses built-in defaults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DAE102_CS1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DAE102_CS2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DAE102_CS3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DAE102_CS4</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DAE102_CS5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DAE102_CS6</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Mr. Ray Leung</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Mr. Ray Leung</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DAE102_CS7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Mr. Ivan Yuen</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DAE102_WT1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DAE102_WT2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DAE102_SW1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DAE102_TW1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DAE102_TW2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DAE102_TW3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mr. Ray Leung</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Mr. Ray Leung</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DAE102_TM1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DAE102_TM2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DAE102_TM3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DAE102_TM4</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Ms. Sasha Cheung</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DAE102_KT1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DAE102_KT2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DAE102_KT3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DAE102_TK1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Ms. Cherry Ip</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DAE102_ST1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Ms. Lee Kit Wan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Ms. Lee Kit Wan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Ms. Lee Kit Wan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Ms. Lee Kit Wan</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DAE102_ST2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DAE102_ST3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Ms. Elise Ye</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DAE102_FL1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Ms. Lee Kit Wan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Ms. Lee Kit Wan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Ms. Lee Kit Wan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Ms. Lee Kit Wan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>